<commit_message>
chore: depurar archivos obsoletos, parches temporales y codigo descontinuado de MODIFICACIONES_PERSONAL
</commit_message>
<xml_diff>
--- a/MODIFICACIONES_SABADOS.xlsx
+++ b/MODIFICACIONES_SABADOS.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J47"/>
+  <dimension ref="A1:K51"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="10.85546875" bestFit="1" customWidth="1" min="2" max="2"/>
@@ -474,6 +474,11 @@
           <t>CLASIFICACION</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>TIMESTAMP</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -2219,7 +2224,6 @@
           <t>2026-07-18</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
           <t>CRISTIAN DAVID ROJAS PRATTO</t>
@@ -2236,10 +2240,194 @@
           <t>AGREGAR</t>
         </is>
       </c>
-      <c r="I47" t="inlineStr"/>
       <c r="J47" t="inlineStr">
         <is>
           <t>Secuencia Normal</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>JULIO 2026</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>CRISTIAN DAVID ROJAS PRATTO</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>CRISTIAN DAVID ROJAS PRATTO</t>
+        </is>
+      </c>
+      <c r="F48" t="n">
+        <v>8</v>
+      </c>
+      <c r="G48" t="n">
+        <v>2</v>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>REEMPLAZAR</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>Cambio de turno con ALEJANDRA SOFIA VENECIA LOPEZ</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>2026-07-01 15:07:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>MAYO 2026</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>ALEJANDRA SOFIA VENECIA LOPEZ</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>ALEJANDRA SOFIA VENECIA LOPEZ</t>
+        </is>
+      </c>
+      <c r="F49" t="n">
+        <v>52</v>
+      </c>
+      <c r="G49" t="n">
+        <v>2</v>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>REEMPLAZAR</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>Cambio de turno con CRISTIAN DAVID ROJAS PRATTO</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>2026-07-01 15:07:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>JULIO 2026</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>DIANA VANESA ROSERO SANTACRUZ</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>DIANA VANESA ROSERO SANTACRUZ</t>
+        </is>
+      </c>
+      <c r="F50" t="n">
+        <v>9</v>
+      </c>
+      <c r="G50" t="n">
+        <v>2</v>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>REEMPLAZAR</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>Cambio de turno con ABRAHAM DAVID MARTINEZ ESCORCIA</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>2026-07-01 15:27:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>MAYO 2026</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>ABRAHAM DAVID MARTINEZ ESCORCIA</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>ABRAHAM DAVID MARTINEZ ESCORCIA</t>
+        </is>
+      </c>
+      <c r="F51" t="n">
+        <v>2</v>
+      </c>
+      <c r="G51" t="n">
+        <v>2</v>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>REEMPLAZAR</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr"/>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>Cambio de turno con DIANA VANESA ROSERO SANTACRUZ</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>2026-07-01 15:27:41</t>
         </is>
       </c>
     </row>

</xml_diff>